<commit_message>
feat: add mobile landscape release package
</commit_message>
<xml_diff>
--- a/单位属性表/20260710.xlsx
+++ b/单位属性表/20260710.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cruelworld\Desktop\小游戏\奇境王冠\单位属性表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B40F875F-7F52-48D8-A245-97EF8C5F4862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5734E66-E5B5-497B-B5D7-17192BFB8570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -873,9 +873,30 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -883,27 +904,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1430,7 +1430,7 @@
         <v>600</v>
       </c>
       <c r="D5" s="2">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E5" s="2">
         <v>60</v>
@@ -1458,22 +1458,22 @@
       </c>
       <c r="M5" s="6">
         <f>D5/G5*1000</f>
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:14" s="6" customFormat="1"/>
     <row r="7" spans="1:14" s="6" customFormat="1"/>
     <row r="8" spans="1:14" s="6" customFormat="1"/>
     <row r="9" spans="1:14" ht="28">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
@@ -1483,17 +1483,17 @@
       <c r="N9" s="6"/>
     </row>
     <row r="10" spans="1:14" ht="20">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="20">
-        <v>7</v>
-      </c>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="14">
+        <v>5</v>
+      </c>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
@@ -1503,17 +1503,17 @@
       <c r="N10" s="6"/>
     </row>
     <row r="11" spans="1:14" ht="19.350000000000001">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21">
-        <v>15</v>
-      </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15">
+        <v>20</v>
+      </c>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
@@ -1523,17 +1523,17 @@
       <c r="N11" s="6"/>
     </row>
     <row r="12" spans="1:14" ht="19.350000000000001">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21">
-        <v>30</v>
-      </c>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15">
+        <v>40</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
@@ -1683,7 +1683,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -1717,7 +1717,7 @@
         <v>22</v>
       </c>
       <c r="B21" s="9">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -1768,56 +1768,56 @@
       <c r="A24" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
     </row>
     <row r="25" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
     </row>
     <row r="26" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12">
+      <c r="B26" s="18"/>
+      <c r="C26" s="18">
         <v>20</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
     </row>
     <row r="27" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12">
-        <v>25</v>
-      </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18">
+        <v>20</v>
+      </c>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
     </row>
     <row r="28" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12">
+      <c r="B28" s="18"/>
+      <c r="C28" s="18">
         <v>1000</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
     </row>
     <row r="29" spans="1:14" s="6" customFormat="1" ht="28">
       <c r="A29" s="16" t="s">
@@ -1832,67 +1832,67 @@
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
     </row>
     <row r="31" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
     </row>
     <row r="32" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12">
-        <v>500</v>
-      </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18">
+        <v>2000</v>
+      </c>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
     </row>
     <row r="33" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12">
-        <v>30</v>
-      </c>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18">
+        <v>200</v>
+      </c>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
     </row>
     <row r="34" spans="1:5" s="6" customFormat="1" ht="44" customHeight="1">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="14" t="s">
+      <c r="B34" s="20"/>
+      <c r="C34" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
     </row>
     <row r="35" spans="1:5" s="6" customFormat="1">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15" t="s">
+      <c r="B35" s="22"/>
+      <c r="C35" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
     </row>
     <row r="36" spans="1:5" s="6" customFormat="1"/>
     <row r="37" spans="1:5" s="6" customFormat="1"/>
@@ -1912,6 +1912,23 @@
     <row r="51" s="6" customFormat="1"/>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C11:G11"/>
@@ -1922,23 +1939,6 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:E35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update balance and pace AI deployments
</commit_message>
<xml_diff>
--- a/单位属性表/20260710.xlsx
+++ b/单位属性表/20260710.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cruelworld\Desktop\小游戏\奇境王冠\单位属性表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5734E66-E5B5-497B-B5D7-17192BFB8570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C384912-48BE-4009-A3FA-B390695AC7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -873,6 +873,24 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -885,25 +903,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1307,7 +1307,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2">
         <v>60</v>
@@ -1349,7 +1349,7 @@
         <v>20</v>
       </c>
       <c r="E3" s="2">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F3" s="2">
         <v>70</v>
@@ -1391,7 +1391,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F4" s="2">
         <v>80</v>
@@ -1433,7 +1433,7 @@
         <v>30</v>
       </c>
       <c r="E5" s="2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F5" s="2">
         <v>100</v>
@@ -1465,15 +1465,15 @@
     <row r="7" spans="1:14" s="6" customFormat="1"/>
     <row r="8" spans="1:14" s="6" customFormat="1"/>
     <row r="9" spans="1:14" ht="28">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
@@ -1483,17 +1483,17 @@
       <c r="N9" s="6"/>
     </row>
     <row r="10" spans="1:14" ht="20">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="14">
+      <c r="B10" s="22"/>
+      <c r="C10" s="20">
         <v>5</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
@@ -1503,17 +1503,17 @@
       <c r="N10" s="6"/>
     </row>
     <row r="11" spans="1:14" ht="19.350000000000001">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21">
         <v>20</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
@@ -1523,17 +1523,17 @@
       <c r="N11" s="6"/>
     </row>
     <row r="12" spans="1:14" ht="19.350000000000001">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15">
+      <c r="B12" s="21"/>
+      <c r="C12" s="21">
         <v>40</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
@@ -1768,56 +1768,56 @@
       <c r="A24" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
     </row>
     <row r="25" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
     </row>
     <row r="26" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18">
+      <c r="B26" s="12"/>
+      <c r="C26" s="12">
         <v>20</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
     </row>
     <row r="27" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18">
+      <c r="B27" s="12"/>
+      <c r="C27" s="12">
         <v>20</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
     </row>
     <row r="28" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18">
+      <c r="B28" s="12"/>
+      <c r="C28" s="12">
         <v>1000</v>
       </c>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
     </row>
     <row r="29" spans="1:14" s="6" customFormat="1" ht="28">
       <c r="A29" s="16" t="s">
@@ -1832,67 +1832,67 @@
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
     </row>
     <row r="31" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
     </row>
     <row r="32" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18">
+      <c r="B32" s="12"/>
+      <c r="C32" s="12">
         <v>2000</v>
       </c>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
     </row>
     <row r="33" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A33" s="18" t="s">
+      <c r="A33" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18">
+      <c r="B33" s="12"/>
+      <c r="C33" s="12">
         <v>200</v>
       </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
     </row>
     <row r="34" spans="1:5" s="6" customFormat="1" ht="44" customHeight="1">
-      <c r="A34" s="20" t="s">
+      <c r="A34" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="21" t="s">
+      <c r="B34" s="13"/>
+      <c r="C34" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
     </row>
     <row r="35" spans="1:5" s="6" customFormat="1">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22" t="s">
+      <c r="B35" s="15"/>
+      <c r="C35" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
     </row>
     <row r="36" spans="1:5" s="6" customFormat="1"/>
     <row r="37" spans="1:5" s="6" customFormat="1"/>
@@ -1912,23 +1912,6 @@
     <row r="51" s="6" customFormat="1"/>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:E25"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C11:G11"/>
@@ -1939,6 +1922,23 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:E35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: shorten cannon turns and sync battle values
</commit_message>
<xml_diff>
--- a/单位属性表/20260710.xlsx
+++ b/单位属性表/20260710.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cruelworld\Desktop\小游戏\奇境王冠\单位属性表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C384912-48BE-4009-A3FA-B390695AC7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC49525A-A8F9-495E-8C35-07D0E459D7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="66">
   <si>
     <t>单位</t>
   </si>
@@ -157,10 +157,6 @@
   </si>
   <si>
     <t>攻击范围（以量城墙的间距为基准）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1/4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -623,6 +619,26 @@
   </si>
   <si>
     <t>防止频繁出现在单一路线爆兵推进</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ai购买药水逻辑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每当ai存够足够购买药水的金币时，就会有30%的概率和购买药水</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ai使用药水逻辑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>随机强化单位</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -735,7 +751,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -790,8 +806,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -825,20 +853,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -873,6 +892,12 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -891,10 +916,7 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1316,7 +1338,7 @@
         <v>200</v>
       </c>
       <c r="H2" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>18</v>
@@ -1325,7 +1347,7 @@
         <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>8</v>
@@ -1343,7 +1365,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="2">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="D3" s="2">
         <v>20</v>
@@ -1358,7 +1380,7 @@
         <v>500</v>
       </c>
       <c r="H3" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>18</v>
@@ -1379,7 +1401,7 @@
     </row>
     <row r="4" spans="1:14" s="6" customFormat="1" ht="30.7">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2">
         <v>10</v>
@@ -1400,7 +1422,7 @@
         <v>800</v>
       </c>
       <c r="H4" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>19</v>
@@ -1409,7 +1431,7 @@
         <v>20</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>11</v>
@@ -1464,18 +1486,22 @@
     <row r="6" spans="1:14" s="6" customFormat="1"/>
     <row r="7" spans="1:14" s="6" customFormat="1"/>
     <row r="8" spans="1:14" s="6" customFormat="1"/>
-    <row r="9" spans="1:14" ht="28">
-      <c r="A9" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
+    <row r="9" spans="1:14" ht="46">
+      <c r="A9" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>63</v>
+      </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
@@ -1483,19 +1509,23 @@
       <c r="N9" s="6"/>
     </row>
     <row r="10" spans="1:14" ht="20">
-      <c r="A10" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="20">
+      <c r="A10" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="23"/>
+      <c r="C10" s="21">
         <v>5</v>
       </c>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>65</v>
+      </c>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
@@ -1503,17 +1533,17 @@
       <c r="N10" s="6"/>
     </row>
     <row r="11" spans="1:14" ht="19.350000000000001">
-      <c r="A11" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21">
+      <c r="A11" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22">
         <v>20</v>
       </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
@@ -1523,17 +1553,17 @@
       <c r="N11" s="6"/>
     </row>
     <row r="12" spans="1:14" ht="19.350000000000001">
-      <c r="A12" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21">
+      <c r="A12" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22">
         <v>40</v>
       </c>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
@@ -1544,25 +1574,25 @@
     </row>
     <row r="13" spans="1:14" ht="15.7">
       <c r="A13" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="C13" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="F13" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="G13" s="10" t="s">
         <v>51</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>52</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
@@ -1574,7 +1604,7 @@
     </row>
     <row r="14" spans="1:14" s="6" customFormat="1" ht="32">
       <c r="A14" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" s="11">
         <v>1</v>
@@ -1592,12 +1622,12 @@
         <v>1</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A15" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="11">
         <v>1.3</v>
@@ -1615,12 +1645,12 @@
         <v>1</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A16" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" s="11">
         <v>2</v>
@@ -1638,12 +1668,12 @@
         <v>2</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:14" s="6" customFormat="1" ht="48">
       <c r="A17" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B17" s="11">
         <v>1.3</v>
@@ -1661,7 +1691,7 @@
         <v>1.3</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -1747,13 +1777,13 @@
       <c r="N22" s="6"/>
     </row>
     <row r="23" spans="1:14" ht="28">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
@@ -1768,131 +1798,131 @@
       <c r="A24" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
+      <c r="B24" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
     </row>
     <row r="25" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
     </row>
     <row r="26" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12">
+      <c r="B26" s="14"/>
+      <c r="C26" s="14">
         <v>20</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
     </row>
     <row r="27" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12">
+      <c r="B27" s="14"/>
+      <c r="C27" s="14">
         <v>20</v>
       </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
     </row>
     <row r="28" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12">
+      <c r="B28" s="14"/>
+      <c r="C28" s="14">
         <v>1000</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:14" s="6" customFormat="1" ht="28">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
     </row>
     <row r="30" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
     </row>
     <row r="32" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12">
+      <c r="B32" s="14"/>
+      <c r="C32" s="14">
         <v>2000</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
     </row>
     <row r="33" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12">
-        <v>200</v>
-      </c>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14">
+        <v>150</v>
+      </c>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
     </row>
     <row r="34" spans="1:5" s="6" customFormat="1" ht="44" customHeight="1">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
     </row>
     <row r="35" spans="1:5" s="6" customFormat="1">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15" t="s">
+      <c r="B35" s="17"/>
+      <c r="C35" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
     </row>
     <row r="36" spans="1:5" s="6" customFormat="1"/>
     <row r="37" spans="1:5" s="6" customFormat="1"/>

</xml_diff>